<commit_message>
Improve performance of some examples (#2137)
* Eliminate inefficiencies in some examples

* Further updates to examples

* Fix tests

* Remove a hackish change
</commit_message>
<xml_diff>
--- a/optaplanner-examples/src/test/resources/org/optaplanner/examples/conferencescheduling/optional/score/testConferenceSchedulingConstraints.xlsx
+++ b/optaplanner-examples/src/test/resources/org/optaplanner/examples/conferencescheduling/optional/score/testConferenceSchedulingConstraints.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="56"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="13"/>
   </bookViews>
   <sheets>
     <sheet name="Configuration" sheetId="1" state="visible" r:id="rId2"/>
@@ -974,7 +974,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C45"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="49.61"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.72"/>
@@ -1422,7 +1422,7 @@
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -1622,7 +1622,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -1805,7 +1805,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -1989,7 +1989,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -2172,7 +2172,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -2255,7 +2255,7 @@
         <v>171</v>
       </c>
       <c r="B4" s="12" t="n">
-        <v>-60</v>
+        <v>-120</v>
       </c>
       <c r="D4" s="7"/>
       <c r="E4" s="7"/>
@@ -2355,7 +2355,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -2541,7 +2541,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -2741,7 +2741,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -2943,7 +2943,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -3147,7 +3147,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -3339,7 +3339,7 @@
     <mergeCell ref="B6:E6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -3354,7 +3354,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.99"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="6.08"/>
@@ -3482,7 +3482,7 @@
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -3668,7 +3668,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -3854,7 +3854,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -4042,7 +4042,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -4243,7 +4243,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -4445,7 +4445,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -4649,7 +4649,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -4858,7 +4858,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -5077,7 +5077,7 @@
     <mergeCell ref="B6:E6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -5279,7 +5279,7 @@
     <mergeCell ref="B6:E6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -5481,7 +5481,7 @@
     <mergeCell ref="B6:E6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -5496,7 +5496,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K10"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="19.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11.52"/>
@@ -5660,7 +5660,7 @@
     <mergeCell ref="I1:K1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -5879,7 +5879,7 @@
     <mergeCell ref="B6:E6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -6081,7 +6081,7 @@
     <mergeCell ref="B6:E6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -6295,7 +6295,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -6509,7 +6509,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -6719,7 +6719,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -6933,7 +6933,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -7151,7 +7151,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -7355,7 +7355,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -7559,7 +7559,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -7763,7 +7763,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -7778,7 +7778,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:P7"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="21.7"/>
@@ -7955,7 +7955,7 @@
     <mergeCell ref="N1:P1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -8159,7 +8159,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -8363,7 +8363,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -8567,7 +8567,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -8773,7 +8773,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -8979,7 +8979,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -9185,7 +9185,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -9391,7 +9391,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -9605,7 +9605,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -9791,7 +9791,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -9981,7 +9981,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -9996,7 +9996,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AE65"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26.95"/>
@@ -12104,7 +12104,7 @@
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -12294,7 +12294,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -12484,7 +12484,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -12674,7 +12674,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -12857,7 +12857,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -13059,7 +13059,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -13261,7 +13261,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -13463,7 +13463,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -13665,7 +13665,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -13849,7 +13849,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -14032,7 +14032,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -14218,7 +14218,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -14403,7 +14403,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>

</xml_diff>